<commit_message>
feat: bo sung day du chi so danh gia Random Forest
</commit_message>
<xml_diff>
--- a/Tho_Churn_Prediction/outputs/churn_model_summary.xlsx
+++ b/Tho_Churn_Prediction/outputs/churn_model_summary.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_quan" sheetId="1" r:id="R38b9828342dc4530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bao_cao_lop" sheetId="2" r:id="R5455cde348f74126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_importance" sheetId="3" r:id="Re3fa044204fc422c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross_validation" sheetId="4" r:id="R34e7231c4c284a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong_quan" sheetId="1" r:id="R9c7aa9723afd41a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bao_cao_lop" sheetId="2" r:id="R85c02117133a4351"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_importance" sheetId="3" r:id="Rb4d170cc1d774607"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross_validation" sheetId="4" r:id="Rb638b199aaf84d70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,12 +68,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -108,7 +113,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -158,6 +163,30 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -347,7 +376,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc01b1adf7b234bf2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb406aacb62d547a2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -598,10 +627,10 @@
         <x:v>Giá trị</x:v>
       </x:c>
       <x:c r="C5" s="22"/>
-      <x:c r="D5" s="6" t="str">
+      <x:c r="D5" s="32" t="str">
         <x:v>Chỉ số tập test</x:v>
       </x:c>
-      <x:c r="E5" s="6" t="str">
+      <x:c r="E5" s="32" t="str">
         <x:v>Kết quả</x:v>
       </x:c>
       <x:c r="F5" s="22"/>
@@ -614,10 +643,10 @@
         <x:v>RandomForestClassifier</x:v>
       </x:c>
       <x:c r="C6" s="22"/>
-      <x:c r="D6" s="22" t="str">
+      <x:c r="D6" s="15" t="str">
         <x:v>Accuracy</x:v>
       </x:c>
-      <x:c r="E6" s="23" t="n">
+      <x:c r="E6" s="33" t="n">
         <x:v>0.8791208791208791</x:v>
       </x:c>
       <x:c r="F6" s="22"/>
@@ -630,10 +659,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="C7" s="22"/>
-      <x:c r="D7" s="22" t="str">
+      <x:c r="D7" s="15" t="str">
         <x:v>Balanced accuracy</x:v>
       </x:c>
-      <x:c r="E7" s="23" t="n">
+      <x:c r="E7" s="33" t="n">
         <x:v>0.6444716533095874</x:v>
       </x:c>
       <x:c r="F7" s="22"/>
@@ -646,11 +675,11 @@
         <x:v>2017-04-01 đến 2018-03-01</x:v>
       </x:c>
       <x:c r="C8" s="22"/>
-      <x:c r="D8" s="22" t="str">
-        <x:v>Macro F1</x:v>
-      </x:c>
-      <x:c r="E8" s="23" t="n">
-        <x:v>0.5888497592677657</x:v>
+      <x:c r="D8" s="15" t="str">
+        <x:v>Macro precision</x:v>
+      </x:c>
+      <x:c r="E8" s="33" t="n">
+        <x:v>0.5715951046585176</x:v>
       </x:c>
       <x:c r="F8" s="22"/>
     </x:row>
@@ -662,11 +691,11 @@
         <x:v>5920</x:v>
       </x:c>
       <x:c r="C9" s="22"/>
-      <x:c r="D9" s="22" t="str">
-        <x:v>Precision lớp quay lại</x:v>
-      </x:c>
-      <x:c r="E9" s="23" t="n">
-        <x:v>0.17829457364341086</x:v>
+      <x:c r="D9" s="15" t="str">
+        <x:v>Macro recall</x:v>
+      </x:c>
+      <x:c r="E9" s="33" t="n">
+        <x:v>0.6444716533095874</x:v>
       </x:c>
       <x:c r="F9" s="22"/>
     </x:row>
@@ -678,11 +707,11 @@
         <x:v>1484</x:v>
       </x:c>
       <x:c r="C10" s="22"/>
-      <x:c r="D10" s="22" t="str">
-        <x:v>Recall lớp quay lại</x:v>
-      </x:c>
-      <x:c r="E10" s="23" t="n">
-        <x:v>0.38333333333333336</x:v>
+      <x:c r="D10" s="15" t="str">
+        <x:v>Macro F1</x:v>
+      </x:c>
+      <x:c r="E10" s="33" t="n">
+        <x:v>0.5888497592677657</x:v>
       </x:c>
       <x:c r="F10" s="22"/>
     </x:row>
@@ -694,11 +723,11 @@
         <x:v>299</x:v>
       </x:c>
       <x:c r="C11" s="22"/>
-      <x:c r="D11" s="22" t="str">
-        <x:v>F1 lớp quay lại</x:v>
-      </x:c>
-      <x:c r="E11" s="23" t="n">
-        <x:v>0.24338624338624337</x:v>
+      <x:c r="D11" s="15" t="str">
+        <x:v>Weighted precision</x:v>
+      </x:c>
+      <x:c r="E11" s="33" t="n">
+        <x:v>0.9250004000676963</x:v>
       </x:c>
       <x:c r="F11" s="22"/>
     </x:row>
@@ -710,11 +739,11 @@
         <x:v>5621</x:v>
       </x:c>
       <x:c r="C12" s="22"/>
-      <x:c r="D12" s="22" t="str">
-        <x:v>Precision lớp churn</x:v>
-      </x:c>
-      <x:c r="E12" s="23" t="n">
-        <x:v>0.9648956356736242</x:v>
+      <x:c r="D12" s="15" t="str">
+        <x:v>Weighted recall</x:v>
+      </x:c>
+      <x:c r="E12" s="33" t="n">
+        <x:v>0.8791208791208791</x:v>
       </x:c>
       <x:c r="F12" s="22"/>
     </x:row>
@@ -726,11 +755,11 @@
         <x:v>4737</x:v>
       </x:c>
       <x:c r="C13" s="22"/>
-      <x:c r="D13" s="22" t="str">
-        <x:v>Recall lớp churn</x:v>
-      </x:c>
-      <x:c r="E13" s="23" t="n">
-        <x:v>0.9056099732858415</x:v>
+      <x:c r="D13" s="15" t="str">
+        <x:v>Weighted F1</x:v>
+      </x:c>
+      <x:c r="E13" s="33" t="n">
+        <x:v>0.8992704840201395</x:v>
       </x:c>
       <x:c r="F13" s="22"/>
     </x:row>
@@ -742,11 +771,11 @@
         <x:v>1187</x:v>
       </x:c>
       <x:c r="C14" s="22"/>
-      <x:c r="D14" s="22" t="str">
-        <x:v>F1 lớp churn</x:v>
-      </x:c>
-      <x:c r="E14" s="23" t="n">
-        <x:v>0.934313275149288</x:v>
+      <x:c r="D14" s="15" t="str">
+        <x:v>Precision lớp quay lại</x:v>
+      </x:c>
+      <x:c r="E14" s="33" t="n">
+        <x:v>0.17829457364341086</x:v>
       </x:c>
       <x:c r="F14" s="22"/>
     </x:row>
@@ -758,11 +787,11 @@
         <x:v>1183</x:v>
       </x:c>
       <x:c r="C15" s="22"/>
-      <x:c r="D15" s="22" t="str">
-        <x:v>ROC-AUC</x:v>
-      </x:c>
-      <x:c r="E15" s="23" t="n">
-        <x:v>0.71675571386168</x:v>
+      <x:c r="D15" s="15" t="str">
+        <x:v>Recall lớp quay lại</x:v>
+      </x:c>
+      <x:c r="E15" s="33" t="n">
+        <x:v>0.38333333333333336</x:v>
       </x:c>
       <x:c r="F15" s="22"/>
     </x:row>
@@ -774,11 +803,11 @@
         <x:v>297</x:v>
       </x:c>
       <x:c r="C16" s="22"/>
-      <x:c r="D16" s="22" t="str">
-        <x:v>Average precision lớp quay lại</x:v>
-      </x:c>
-      <x:c r="E16" s="23" t="n">
-        <x:v>0.21973234417038148</x:v>
+      <x:c r="D16" s="15" t="str">
+        <x:v>F1 lớp quay lại</x:v>
+      </x:c>
+      <x:c r="E16" s="33" t="n">
+        <x:v>0.24338624338624337</x:v>
       </x:c>
       <x:c r="F16" s="22"/>
     </x:row>
@@ -790,11 +819,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C17" s="22"/>
-      <x:c r="D17" s="22" t="str">
-        <x:v>Macro F1 mốc đoán toàn bộ churn</x:v>
-      </x:c>
-      <x:c r="E17" s="23" t="n">
-        <x:v>0.486990459670425</x:v>
+      <x:c r="D17" s="15" t="str">
+        <x:v>F1 lớp churn</x:v>
+      </x:c>
+      <x:c r="E17" s="33" t="n">
+        <x:v>0.934313275149288</x:v>
       </x:c>
       <x:c r="F17" s="22"/>
     </x:row>
@@ -806,16 +835,24 @@
         <x:v>0.5700000000000002</x:v>
       </x:c>
       <x:c r="C18" s="22"/>
-      <x:c r="D18" s="22"/>
-      <x:c r="E18" s="22"/>
+      <x:c r="D18" s="15" t="str">
+        <x:v>ROC-AUC</x:v>
+      </x:c>
+      <x:c r="E18" s="33" t="n">
+        <x:v>0.71675571386168</x:v>
+      </x:c>
       <x:c r="F18" s="22"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22"/>
       <x:c r="B19" s="22"/>
       <x:c r="C19" s="22"/>
-      <x:c r="D19" s="22"/>
-      <x:c r="E19" s="22"/>
+      <x:c r="D19" s="15" t="str">
+        <x:v>Average precision lớp quay lại</x:v>
+      </x:c>
+      <x:c r="E19" s="33" t="n">
+        <x:v>0.21973234417038148</x:v>
+      </x:c>
       <x:c r="F19" s="22"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
@@ -950,7 +987,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="27" t="str">
-        <x:v>Lưu ý: dữ liệu vẫn mất cân bằng. Đọc accuracy cùng balanced accuracy, macro F1 và kết quả từng lớp.</x:v>
+        <x:v>Lưu ý: dữ liệu mất cân bằng. Cần đọc macro avg, weighted avg và kết quả từng lớp cùng nhau.</x:v>
       </x:c>
       <x:c r="B30" s="22"/>
       <x:c r="C30" s="22"/>
@@ -980,166 +1017,169 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="3" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="35"/>
+      <x:c r="B1" s="35"/>
+      <x:c r="C1" s="35"/>
+      <x:c r="D1" s="35"/>
+      <x:c r="E1" s="35"/>
+      <x:c r="F1" s="35"/>
+      <x:c r="G1" s="35"/>
+      <x:c r="H1" s="35"/>
+      <x:c r="I1" s="35"/>
+    </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="20" t="str">
-        <x:v>Kết quả theo từng lớp</x:v>
-      </x:c>
-      <x:c r="B2" s="20"/>
-      <x:c r="C2" s="20"/>
-      <x:c r="D2" s="20"/>
-      <x:c r="E2" s="20"/>
-      <x:c r="F2" s="20"/>
-      <x:c r="G2" s="20"/>
-      <x:c r="H2" s="20"/>
-      <x:c r="I2" s="20"/>
+        <x:v>Báo cáo phân loại train và test</x:v>
+      </x:c>
+      <x:c r="B2" s="35"/>
+      <x:c r="C2" s="35"/>
+      <x:c r="D2" s="35"/>
+      <x:c r="E2" s="35"/>
+      <x:c r="F2" s="35"/>
+      <x:c r="G2" s="35"/>
+      <x:c r="H2" s="35"/>
+      <x:c r="I2" s="35"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="21" t="str">
         <x:v>Lớp 0 là khách quay lại mua. Lớp 1 là churn proxy trong 180 ngày.</x:v>
       </x:c>
-      <x:c r="B3" s="22"/>
-      <x:c r="C3" s="22"/>
-      <x:c r="D3" s="22"/>
-      <x:c r="E3" s="22"/>
-      <x:c r="F3" s="22"/>
-      <x:c r="G3" s="22"/>
-      <x:c r="H3" s="22"/>
-      <x:c r="I3" s="22"/>
+      <x:c r="B3" s="35"/>
+      <x:c r="C3" s="35"/>
+      <x:c r="D3" s="35"/>
+      <x:c r="E3" s="35"/>
+      <x:c r="F3" s="35"/>
+      <x:c r="G3" s="35"/>
+      <x:c r="H3" s="35"/>
+      <x:c r="I3" s="35"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="22"/>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="22"/>
-      <x:c r="E4" s="22"/>
-      <x:c r="F4" s="22"/>
-      <x:c r="G4" s="22"/>
-      <x:c r="H4" s="22"/>
-      <x:c r="I4" s="22"/>
+      <x:c r="A4" s="35"/>
+      <x:c r="B4" s="35"/>
+      <x:c r="C4" s="35"/>
+      <x:c r="D4" s="35"/>
+      <x:c r="E4" s="35"/>
+      <x:c r="F4" s="35"/>
+      <x:c r="G4" s="35"/>
+      <x:c r="H4" s="35"/>
+      <x:c r="I4" s="35"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
-      <x:c r="A5" s="6" t="str">
-        <x:v>﻿class</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="str">
+      <x:c r="A5" s="20" t="str">
+        <x:v>Tập test</x:v>
+      </x:c>
+      <x:c r="B5" s="35"/>
+      <x:c r="C5" s="35"/>
+      <x:c r="D5" s="35"/>
+      <x:c r="E5" s="35"/>
+      <x:c r="F5" s="35"/>
+      <x:c r="G5" s="35"/>
+      <x:c r="H5" s="35"/>
+      <x:c r="I5" s="35"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="32" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="B6" s="32" t="str">
         <x:v>precision</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="str">
+      <x:c r="C6" s="32" t="str">
         <x:v>recall</x:v>
       </x:c>
-      <x:c r="D5" s="6" t="str">
+      <x:c r="D6" s="32" t="str">
         <x:v>f1-score</x:v>
       </x:c>
-      <x:c r="E5" s="6" t="str">
+      <x:c r="E6" s="32" t="str">
         <x:v>support</x:v>
       </x:c>
-      <x:c r="F5" s="22"/>
-      <x:c r="G5" s="6" t="str">
+      <x:c r="F6" s="35"/>
+      <x:c r="G6" s="32" t="str">
         <x:v>Thực tế / Dự đoán</x:v>
       </x:c>
-      <x:c r="H5" s="6" t="str">
+      <x:c r="H6" s="32" t="str">
         <x:v>Quay lại</x:v>
       </x:c>
-      <x:c r="I5" s="6" t="str">
+      <x:c r="I6" s="32" t="str">
         <x:v>Churn</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="22" t="str">
-        <x:v>Quay_lai_0</x:v>
-      </x:c>
-      <x:c r="B6" s="23" t="n">
-        <x:v>0.17829457364341086</x:v>
-      </x:c>
-      <x:c r="C6" s="23" t="n">
-        <x:v>0.38333333333333336</x:v>
-      </x:c>
-      <x:c r="D6" s="23" t="n">
-        <x:v>0.24338624338624337</x:v>
-      </x:c>
-      <x:c r="E6" s="25" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F6" s="22"/>
-      <x:c r="G6" s="22" t="str">
-        <x:v>Quay lại</x:v>
-      </x:c>
-      <x:c r="H6" s="25" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="I6" s="25" t="n">
-        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="str">
-        <x:v>Churn_1</x:v>
-      </x:c>
-      <x:c r="B7" s="23" t="n">
-        <x:v>0.9648956356736242</x:v>
-      </x:c>
-      <x:c r="C7" s="23" t="n">
-        <x:v>0.9056099732858415</x:v>
-      </x:c>
-      <x:c r="D7" s="23" t="n">
-        <x:v>0.934313275149288</x:v>
-      </x:c>
-      <x:c r="E7" s="25" t="n">
-        <x:v>1123</x:v>
+        <x:v>Quay_lai_0</x:v>
+      </x:c>
+      <x:c r="B7" s="36" t="n">
+        <x:v>0.17829457364341086</x:v>
+      </x:c>
+      <x:c r="C7" s="36" t="n">
+        <x:v>0.38333333333333336</x:v>
+      </x:c>
+      <x:c r="D7" s="36" t="n">
+        <x:v>0.24338624338624337</x:v>
+      </x:c>
+      <x:c r="E7" s="37" t="n">
+        <x:v>60</x:v>
       </x:c>
       <x:c r="F7" s="22"/>
       <x:c r="G7" s="22" t="str">
-        <x:v>Churn</x:v>
-      </x:c>
-      <x:c r="H7" s="25" t="n">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="I7" s="25" t="n">
-        <x:v>1017</x:v>
+        <x:v>Quay lại</x:v>
+      </x:c>
+      <x:c r="H7" s="37" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I7" s="37" t="n">
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22" t="str">
-        <x:v>accuracy</x:v>
-      </x:c>
-      <x:c r="B8" s="23"/>
-      <x:c r="C8" s="23"/>
-      <x:c r="D8" s="23" t="n">
-        <x:v>0.8791208791208791</x:v>
-      </x:c>
-      <x:c r="E8" s="25" t="n">
-        <x:v>1183</x:v>
+        <x:v>Churn_1</x:v>
+      </x:c>
+      <x:c r="B8" s="36" t="n">
+        <x:v>0.9648956356736242</x:v>
+      </x:c>
+      <x:c r="C8" s="36" t="n">
+        <x:v>0.9056099732858415</x:v>
+      </x:c>
+      <x:c r="D8" s="36" t="n">
+        <x:v>0.934313275149288</x:v>
+      </x:c>
+      <x:c r="E8" s="37" t="n">
+        <x:v>1123</x:v>
       </x:c>
       <x:c r="F8" s="22"/>
-      <x:c r="G8" s="22"/>
-      <x:c r="H8" s="22"/>
-      <x:c r="I8" s="22"/>
+      <x:c r="G8" s="22" t="str">
+        <x:v>Churn</x:v>
+      </x:c>
+      <x:c r="H8" s="37" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="I8" s="37" t="n">
+        <x:v>1017</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="22" t="str">
-        <x:v>macro avg</x:v>
-      </x:c>
-      <x:c r="B9" s="23" t="n">
-        <x:v>0.5715951046585176</x:v>
-      </x:c>
-      <x:c r="C9" s="23" t="n">
-        <x:v>0.6444716533095874</x:v>
-      </x:c>
-      <x:c r="D9" s="23" t="n">
-        <x:v>0.5888497592677657</x:v>
-      </x:c>
-      <x:c r="E9" s="25" t="n">
+        <x:v>accuracy</x:v>
+      </x:c>
+      <x:c r="B9" s="36"/>
+      <x:c r="C9" s="36"/>
+      <x:c r="D9" s="36" t="n">
+        <x:v>0.8791208791208791</x:v>
+      </x:c>
+      <x:c r="E9" s="37" t="n">
         <x:v>1183</x:v>
       </x:c>
       <x:c r="F9" s="22"/>
@@ -1149,18 +1189,18 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22" t="str">
-        <x:v>weighted avg</x:v>
-      </x:c>
-      <x:c r="B10" s="23" t="n">
-        <x:v>0.9250004000676963</x:v>
-      </x:c>
-      <x:c r="C10" s="23" t="n">
-        <x:v>0.8791208791208791</x:v>
-      </x:c>
-      <x:c r="D10" s="23" t="n">
-        <x:v>0.8992704840201395</x:v>
-      </x:c>
-      <x:c r="E10" s="25" t="n">
+        <x:v>macro avg</x:v>
+      </x:c>
+      <x:c r="B10" s="36" t="n">
+        <x:v>0.5715951046585176</x:v>
+      </x:c>
+      <x:c r="C10" s="36" t="n">
+        <x:v>0.6444716533095874</x:v>
+      </x:c>
+      <x:c r="D10" s="36" t="n">
+        <x:v>0.5888497592677657</x:v>
+      </x:c>
+      <x:c r="E10" s="37" t="n">
         <x:v>1183</x:v>
       </x:c>
       <x:c r="F10" s="22"/>
@@ -1169,15 +1209,224 @@
       <x:c r="I10" s="22"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="22"/>
-      <x:c r="B11" s="22"/>
-      <x:c r="C11" s="22"/>
-      <x:c r="D11" s="22"/>
-      <x:c r="E11" s="22"/>
+      <x:c r="A11" s="22" t="str">
+        <x:v>weighted avg</x:v>
+      </x:c>
+      <x:c r="B11" s="36" t="n">
+        <x:v>0.9250004000676963</x:v>
+      </x:c>
+      <x:c r="C11" s="36" t="n">
+        <x:v>0.8791208791208791</x:v>
+      </x:c>
+      <x:c r="D11" s="36" t="n">
+        <x:v>0.8992704840201395</x:v>
+      </x:c>
+      <x:c r="E11" s="37" t="n">
+        <x:v>1183</x:v>
+      </x:c>
       <x:c r="F11" s="22"/>
       <x:c r="G11" s="22"/>
       <x:c r="H11" s="22"/>
       <x:c r="I11" s="22"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="22"/>
+      <x:c r="B12" s="22"/>
+      <x:c r="C12" s="22"/>
+      <x:c r="D12" s="22"/>
+      <x:c r="E12" s="22"/>
+      <x:c r="F12" s="22"/>
+      <x:c r="G12" s="22"/>
+      <x:c r="H12" s="22"/>
+      <x:c r="I12" s="22"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="str">
+        <x:v>Tập train</x:v>
+      </x:c>
+      <x:c r="B13" s="22"/>
+      <x:c r="C13" s="22"/>
+      <x:c r="D13" s="22"/>
+      <x:c r="E13" s="22"/>
+      <x:c r="F13" s="22"/>
+      <x:c r="G13" s="22"/>
+      <x:c r="H13" s="22"/>
+      <x:c r="I13" s="22"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="32" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="B14" s="32" t="str">
+        <x:v>precision</x:v>
+      </x:c>
+      <x:c r="C14" s="32" t="str">
+        <x:v>recall</x:v>
+      </x:c>
+      <x:c r="D14" s="32" t="str">
+        <x:v>f1-score</x:v>
+      </x:c>
+      <x:c r="E14" s="32" t="str">
+        <x:v>support</x:v>
+      </x:c>
+      <x:c r="F14" s="22"/>
+      <x:c r="G14" s="32" t="str">
+        <x:v>Thực tế / Dự đoán</x:v>
+      </x:c>
+      <x:c r="H14" s="32" t="str">
+        <x:v>Quay lại</x:v>
+      </x:c>
+      <x:c r="I14" s="32" t="str">
+        <x:v>Churn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="22" t="str">
+        <x:v>Quay_lai_0</x:v>
+      </x:c>
+      <x:c r="B15" s="36" t="n">
+        <x:v>0.5207373271889401</x:v>
+      </x:c>
+      <x:c r="C15" s="36" t="n">
+        <x:v>0.9456066945606695</x:v>
+      </x:c>
+      <x:c r="D15" s="36" t="n">
+        <x:v>0.6716196136701337</x:v>
+      </x:c>
+      <x:c r="E15" s="37" t="n">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="F15" s="22"/>
+      <x:c r="G15" s="22" t="str">
+        <x:v>Quay lại</x:v>
+      </x:c>
+      <x:c r="H15" s="37" t="n">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="I15" s="37" t="n">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="22" t="str">
+        <x:v>Churn_1</x:v>
+      </x:c>
+      <x:c r="B16" s="36" t="n">
+        <x:v>0.9969788519637462</x:v>
+      </x:c>
+      <x:c r="C16" s="36" t="n">
+        <x:v>0.953757225433526</x:v>
+      </x:c>
+      <x:c r="D16" s="36" t="n">
+        <x:v>0.9748892171344166</x:v>
+      </x:c>
+      <x:c r="E16" s="37" t="n">
+        <x:v>4498</x:v>
+      </x:c>
+      <x:c r="F16" s="22"/>
+      <x:c r="G16" s="22" t="str">
+        <x:v>Churn</x:v>
+      </x:c>
+      <x:c r="H16" s="37" t="n">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="I16" s="37" t="n">
+        <x:v>4290</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="22" t="str">
+        <x:v>accuracy</x:v>
+      </x:c>
+      <x:c r="B17" s="36"/>
+      <x:c r="C17" s="36"/>
+      <x:c r="D17" s="36" t="n">
+        <x:v>0.9533459995777919</x:v>
+      </x:c>
+      <x:c r="E17" s="37" t="n">
+        <x:v>4737</x:v>
+      </x:c>
+      <x:c r="F17" s="22"/>
+      <x:c r="G17" s="22"/>
+      <x:c r="H17" s="22"/>
+      <x:c r="I17" s="22"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="str">
+        <x:v>macro avg</x:v>
+      </x:c>
+      <x:c r="B18" s="36" t="n">
+        <x:v>0.7588580895763432</x:v>
+      </x:c>
+      <x:c r="C18" s="36" t="n">
+        <x:v>0.9496819599970978</x:v>
+      </x:c>
+      <x:c r="D18" s="36" t="n">
+        <x:v>0.8232544154022752</x:v>
+      </x:c>
+      <x:c r="E18" s="37" t="n">
+        <x:v>4737</x:v>
+      </x:c>
+      <x:c r="F18" s="22"/>
+      <x:c r="G18" s="22"/>
+      <x:c r="H18" s="22"/>
+      <x:c r="I18" s="22"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="22" t="str">
+        <x:v>weighted avg</x:v>
+      </x:c>
+      <x:c r="B19" s="36" t="n">
+        <x:v>0.9729506221936008</x:v>
+      </x:c>
+      <x:c r="C19" s="36" t="n">
+        <x:v>0.9533459995777919</x:v>
+      </x:c>
+      <x:c r="D19" s="36" t="n">
+        <x:v>0.9595880908460561</x:v>
+      </x:c>
+      <x:c r="E19" s="37" t="n">
+        <x:v>4737</x:v>
+      </x:c>
+      <x:c r="F19" s="22"/>
+      <x:c r="G19" s="22"/>
+      <x:c r="H19" s="22"/>
+      <x:c r="I19" s="22"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="22"/>
+      <x:c r="B20" s="22"/>
+      <x:c r="C20" s="22"/>
+      <x:c r="D20" s="22"/>
+      <x:c r="E20" s="22"/>
+      <x:c r="F20" s="22"/>
+      <x:c r="G20" s="22"/>
+      <x:c r="H20" s="22"/>
+      <x:c r="I20" s="22"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="27" t="str">
+        <x:v>Weighted avg bị ảnh hưởng nhiều bởi lớp churn. Macro avg cho hai lớp trọng số như nhau.</x:v>
+      </x:c>
+      <x:c r="B21" s="22"/>
+      <x:c r="C21" s="22"/>
+      <x:c r="D21" s="22"/>
+      <x:c r="E21" s="22"/>
+      <x:c r="F21" s="22"/>
+      <x:c r="G21" s="22"/>
+      <x:c r="H21" s="22"/>
+      <x:c r="I21" s="22"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="35"/>
+      <x:c r="B22" s="35"/>
+      <x:c r="C22" s="35"/>
+      <x:c r="D22" s="35"/>
+      <x:c r="E22" s="35"/>
+      <x:c r="F22" s="35"/>
+      <x:c r="G22" s="35"/>
+      <x:c r="H22" s="35"/>
+      <x:c r="I22" s="35"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1243,7 +1492,7 @@
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>﻿feature</x:v>
+        <x:v>feature</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
         <x:v>importance</x:v>
@@ -2107,7 +2356,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3879cb0eacb4e82"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2362802274ec481f"/>
 </x:worksheet>
 </file>
 

</xml_diff>